<commit_message>
Update 972400 - MSCI Spain Index .xlsx
</commit_message>
<xml_diff>
--- a/data/972400 - MSCI Spain Index .xlsx
+++ b/data/972400 - MSCI Spain Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7129" uniqueCount="7128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7153" uniqueCount="7152">
   <si>
     <t>Index Level:</t>
   </si>
@@ -21395,6 +21395,78 @@
   </si>
   <si>
     <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -21780,7 +21852,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E7113"/>
+  <dimension ref="A3:E7137"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -78721,6 +78793,198 @@
         <v>7304.288027</v>
       </c>
     </row>
+    <row r="7114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7114" t="s">
+        <v>7128</v>
+      </c>
+      <c r="B7114">
+        <v>7355.211236</v>
+      </c>
+    </row>
+    <row r="7115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7115" t="s">
+        <v>7129</v>
+      </c>
+      <c r="B7115">
+        <v>7427.077327</v>
+      </c>
+    </row>
+    <row r="7116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7116" t="s">
+        <v>7130</v>
+      </c>
+      <c r="B7116">
+        <v>7715.395857</v>
+      </c>
+    </row>
+    <row r="7117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7117" t="s">
+        <v>7131</v>
+      </c>
+      <c r="B7117">
+        <v>7659.584515</v>
+      </c>
+    </row>
+    <row r="7118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7118" t="s">
+        <v>7132</v>
+      </c>
+      <c r="B7118">
+        <v>7659.584515</v>
+      </c>
+    </row>
+    <row r="7119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7119" t="s">
+        <v>7133</v>
+      </c>
+      <c r="B7119">
+        <v>7653.948079</v>
+      </c>
+    </row>
+    <row r="7120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7120" t="s">
+        <v>7134</v>
+      </c>
+      <c r="B7120">
+        <v>7639.501353</v>
+      </c>
+    </row>
+    <row r="7121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7121" t="s">
+        <v>7135</v>
+      </c>
+      <c r="B7121">
+        <v>8036.120272</v>
+      </c>
+    </row>
+    <row r="7122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7122" t="s">
+        <v>7136</v>
+      </c>
+      <c r="B7122">
+        <v>8012.754611</v>
+      </c>
+    </row>
+    <row r="7123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7123" t="s">
+        <v>7137</v>
+      </c>
+      <c r="B7123">
+        <v>8088.905785</v>
+      </c>
+    </row>
+    <row r="7124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7124" t="s">
+        <v>7138</v>
+      </c>
+      <c r="B7124">
+        <v>7997.129009</v>
+      </c>
+    </row>
+    <row r="7125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7125" t="s">
+        <v>7139</v>
+      </c>
+      <c r="B7125">
+        <v>8182.629108</v>
+      </c>
+    </row>
+    <row r="7126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7126" t="s">
+        <v>7140</v>
+      </c>
+      <c r="B7126">
+        <v>8126.263307</v>
+      </c>
+    </row>
+    <row r="7127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7127" t="s">
+        <v>7141</v>
+      </c>
+      <c r="B7127">
+        <v>8066.31791</v>
+      </c>
+    </row>
+    <row r="7128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7128" t="s">
+        <v>7142</v>
+      </c>
+      <c r="B7128">
+        <v>8272.732238</v>
+      </c>
+    </row>
+    <row r="7129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7129" t="s">
+        <v>7143</v>
+      </c>
+      <c r="B7129">
+        <v>8131.361629</v>
+      </c>
+    </row>
+    <row r="7130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7130" t="s">
+        <v>7144</v>
+      </c>
+      <c r="B7130">
+        <v>8065.76014</v>
+      </c>
+    </row>
+    <row r="7131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7131" t="s">
+        <v>7145</v>
+      </c>
+      <c r="B7131">
+        <v>7986.932101</v>
+      </c>
+    </row>
+    <row r="7132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7132" t="s">
+        <v>7146</v>
+      </c>
+      <c r="B7132">
+        <v>7919.7163</v>
+      </c>
+    </row>
+    <row r="7133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7133" t="s">
+        <v>7147</v>
+      </c>
+      <c r="B7133">
+        <v>7840.262132</v>
+      </c>
+    </row>
+    <row r="7134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7134" t="s">
+        <v>7148</v>
+      </c>
+      <c r="B7134">
+        <v>7870.959441</v>
+      </c>
+    </row>
+    <row r="7135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7135" t="s">
+        <v>7149</v>
+      </c>
+      <c r="B7135">
+        <v>7895.957802</v>
+      </c>
+    </row>
+    <row r="7136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7136" t="s">
+        <v>7150</v>
+      </c>
+      <c r="B7136">
+        <v>7854.95267</v>
+      </c>
+    </row>
+    <row r="7137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7137" t="s">
+        <v>7151</v>
+      </c>
+      <c r="B7137">
+        <v>7945.871691</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>